<commit_message>
added repositories and services and test files for it
</commit_message>
<xml_diff>
--- a/question_bank/C1.xlsx
+++ b/question_bank/C1.xlsx
@@ -568,12 +568,12 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Evaluator Keywords</t>
+          <t>Keywords</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Evaluator Notes</t>
+          <t>Expected Answer Notes</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">

</xml_diff>